<commit_message>
configuration et test du swagger
</commit_message>
<xml_diff>
--- a/Docs/CDC et ToDo/Estimation_Nexora.xlsx
+++ b/Docs/CDC et ToDo/Estimation_Nexora.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harim\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\harim\OneDrive\Documents\GitHub\Gestion-de-recherche-en-Biodiversite\Docs\CDC et ToDo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{706FDE93-5E37-490E-8822-3B9CAF8A32BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FD32F6F-656E-405C-A86B-33EA0BB78F94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>

</xml_diff>